<commit_message>
Check swaps against each dish's ingredients; file low fat cream as cream and sour cream dip as curd
</commit_message>
<xml_diff>
--- a/data/amma_ji_recipes.xlsx
+++ b/data/amma_ji_recipes.xlsx
@@ -77297,7 +77297,7 @@
       </c>
       <c r="B1904" t="inlineStr">
         <is>
-          <t>cheese</t>
+          <t>cream</t>
         </is>
       </c>
       <c r="C1904" t="inlineStr">
@@ -77318,7 +77318,11 @@
           <t>no</t>
         </is>
       </c>
-      <c r="G1904" t="inlineStr"/>
+      <c r="G1904" t="inlineStr">
+        <is>
+          <t>milk, skip</t>
+        </is>
+      </c>
     </row>
     <row r="1905">
       <c r="A1905" t="inlineStr">

</xml_diff>